<commit_message>
feat:在 Settings 页签新增了 "Auto-hide on focus lost" 开关，默认开启。
关掉之后，切到别的窗口系统面板就不会自动收起了。
</commit_message>
<xml_diff>
--- a/luban-excels/xlsx/Main.xlsx
+++ b/luban-excels/xlsx/Main.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="29868" windowHeight="13451"/>
+    <workbookView windowWidth="29868" windowHeight="13451" activeTab="7"/>
   </bookViews>
   <sheets>
     <sheet name="Item" sheetId="1" r:id="rId1"/>
@@ -14,6 +14,7 @@
     <sheet name="GameDevelopConfig" sheetId="5" r:id="rId5"/>
     <sheet name="PayTable" sheetId="6" r:id="rId6"/>
     <sheet name="RarityUI" sheetId="7" r:id="rId7"/>
+    <sheet name="TabGroup" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1066" uniqueCount="604">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1100" uniqueCount="615">
   <si>
     <t>##var</t>
   </si>
@@ -107,7 +108,7 @@
     <t>内部名称方便记忆</t>
   </si>
   <si>
-    <t>排序权重，数字越大约靠前</t>
+    <t>排序权重，数字越小约靠前</t>
   </si>
   <si>
     <t>盲盒权重</t>
@@ -1455,6 +1456,9 @@
     <t>North Korea国际制裁/政治</t>
   </si>
   <si>
+    <t>卡面</t>
+  </si>
+  <si>
     <t>SY</t>
   </si>
   <si>
@@ -1849,6 +1853,36 @@
   </si>
   <si>
     <t>UI\ItemUI\Plate_Special2.png</t>
+  </si>
+  <si>
+    <t>TabName</t>
+  </si>
+  <si>
+    <t>*ItemTypeList</t>
+  </si>
+  <si>
+    <t>list,EItemType</t>
+  </si>
+  <si>
+    <t>包含类型</t>
+  </si>
+  <si>
+    <t>在标签栏的顺序</t>
+  </si>
+  <si>
+    <t>Hat</t>
+  </si>
+  <si>
+    <t>Eye</t>
+  </si>
+  <si>
+    <t>Player</t>
+  </si>
+  <si>
+    <t>Theme</t>
+  </si>
+  <si>
+    <t>Card</t>
   </si>
 </sst>
 </file>
@@ -2479,11 +2513,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -3117,7 +3151,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" s="3" customFormat="1" ht="121.8" spans="1:16">
+    <row r="3" s="4" customFormat="1" ht="121.8" spans="1:16">
       <c r="A3" s="2" t="s">
         <v>22</v>
       </c>
@@ -3126,28 +3160,28 @@
       <c r="D3" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="H3" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="I3" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="J3" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="K3" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="L3" s="3" t="s">
+      <c r="L3" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="M3" s="3" t="s">
+      <c r="M3" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="N3" s="3" t="s">
+      <c r="N3" s="4" t="s">
         <v>31</v>
       </c>
     </row>
@@ -6613,303 +6647,312 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:13">
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="3" t="s">
         <v>425</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="3">
         <v>1</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="3" t="s">
         <v>426</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4" t="s">
+      <c r="I2" s="3"/>
+      <c r="J2" s="3" t="s">
         <v>427</v>
       </c>
-      <c r="K2" s="4" t="s">
+      <c r="K2" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="L2" s="4">
+      <c r="L2" s="3">
         <v>1</v>
       </c>
-      <c r="M2" s="4" t="s">
+      <c r="M2" s="3" t="s">
         <v>428</v>
       </c>
     </row>
     <row r="3" spans="2:13">
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="3" t="s">
         <v>429</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="3">
         <v>2</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="3" t="s">
         <v>430</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4" t="s">
+      <c r="I3" s="3"/>
+      <c r="J3" s="3" t="s">
         <v>431</v>
       </c>
-      <c r="K3" s="4" t="s">
+      <c r="K3" s="3" t="s">
         <v>432</v>
       </c>
-      <c r="L3" s="4">
+      <c r="L3" s="3">
         <v>2</v>
       </c>
-      <c r="M3" s="4" t="s">
+      <c r="M3" s="3" t="s">
         <v>433</v>
       </c>
     </row>
     <row r="4" spans="2:13">
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="3" t="s">
         <v>434</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="3">
         <v>3</v>
       </c>
-      <c r="G4" s="4" t="s">
+      <c r="G4" s="3" t="s">
         <v>435</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="H4" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4" t="s">
+      <c r="I4" s="3"/>
+      <c r="J4" s="3" t="s">
         <v>436</v>
       </c>
-      <c r="K4" s="4" t="s">
+      <c r="K4" s="3" t="s">
         <v>437</v>
       </c>
-      <c r="L4" s="4">
+      <c r="L4" s="3">
         <v>4</v>
       </c>
-      <c r="M4" s="4" t="s">
+      <c r="M4" s="3" t="s">
         <v>438</v>
       </c>
     </row>
     <row r="5" spans="2:13">
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="3" t="s">
         <v>439</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="3">
         <v>4</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="3" t="s">
         <v>440</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" s="3" t="s">
         <v>366</v>
       </c>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4" t="s">
+      <c r="I5" s="3"/>
+      <c r="J5" s="3" t="s">
         <v>441</v>
       </c>
-      <c r="K5" s="4" t="s">
+      <c r="K5" s="3" t="s">
         <v>442</v>
       </c>
-      <c r="L5" s="4">
+      <c r="L5" s="3">
         <v>8</v>
       </c>
-      <c r="M5" s="4" t="s">
+      <c r="M5" s="3" t="s">
         <v>443</v>
       </c>
     </row>
     <row r="6" spans="2:13">
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="3" t="s">
         <v>444</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D6" s="3">
         <v>5</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="G6" s="3" t="s">
         <v>445</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" s="3" t="s">
         <v>446</v>
       </c>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4" t="s">
+      <c r="I6" s="3"/>
+      <c r="J6" s="3" t="s">
         <v>447</v>
       </c>
-      <c r="K6" s="4" t="s">
+      <c r="K6" s="3" t="s">
         <v>448</v>
       </c>
-      <c r="L6" s="4">
+      <c r="L6" s="3">
         <v>16</v>
       </c>
-      <c r="M6" s="4" t="s">
+      <c r="M6" s="3" t="s">
         <v>449</v>
       </c>
     </row>
     <row r="7" spans="2:13">
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>450</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D7" s="3">
         <v>6</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7" s="3" t="s">
         <v>451</v>
       </c>
-      <c r="H7" s="4" t="s">
+      <c r="H7" s="3" t="s">
         <v>452</v>
       </c>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4" t="s">
+      <c r="I7" s="3"/>
+      <c r="J7" s="3" t="s">
         <v>453</v>
       </c>
-      <c r="K7" s="4" t="s">
+      <c r="K7" s="3" t="s">
         <v>454</v>
       </c>
-      <c r="L7" s="4">
+      <c r="L7" s="3">
         <v>32</v>
       </c>
-      <c r="M7" s="4" t="s">
+      <c r="M7" s="3" t="s">
         <v>455</v>
       </c>
     </row>
     <row r="8" spans="2:13">
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>249</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="3" t="s">
         <v>456</v>
       </c>
-      <c r="D8" s="4">
+      <c r="D8" s="3">
         <v>7</v>
       </c>
-      <c r="J8" s="4" t="s">
+      <c r="J8" s="3" t="s">
         <v>457</v>
       </c>
-      <c r="K8" s="4" t="s">
+      <c r="K8" s="3" t="s">
         <v>458</v>
       </c>
-      <c r="L8" s="4">
+      <c r="L8" s="3">
         <v>64</v>
       </c>
-      <c r="M8" s="4" t="s">
+      <c r="M8" s="3" t="s">
         <v>459</v>
       </c>
     </row>
     <row r="9" spans="2:13">
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="3" t="s">
         <v>321</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="3" t="s">
         <v>460</v>
       </c>
-      <c r="D9" s="4">
+      <c r="D9" s="3">
         <v>8</v>
       </c>
-      <c r="J9" s="4" t="s">
+      <c r="J9" s="3" t="s">
         <v>461</v>
       </c>
-      <c r="K9" s="4" t="s">
+      <c r="K9" s="3" t="s">
         <v>462</v>
       </c>
-      <c r="L9" s="4">
+      <c r="L9" s="3">
         <v>128</v>
       </c>
-      <c r="M9" s="4" t="s">
+      <c r="M9" s="3" t="s">
         <v>463</v>
       </c>
     </row>
     <row r="10" spans="2:13">
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="3" t="s">
         <v>365</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="3" t="s">
         <v>464</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D10" s="3">
         <v>9</v>
       </c>
-      <c r="J10" s="4" t="s">
+      <c r="J10" s="3" t="s">
         <v>465</v>
       </c>
-      <c r="K10" s="4" t="s">
+      <c r="K10" s="3" t="s">
         <v>466</v>
       </c>
-      <c r="L10" s="4">
+      <c r="L10" s="3">
         <v>256</v>
       </c>
-      <c r="M10" s="4" t="s">
+      <c r="M10" s="3" t="s">
         <v>467</v>
       </c>
     </row>
     <row r="11" spans="2:13">
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="3" t="s">
         <v>413</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="3" t="s">
         <v>468</v>
       </c>
-      <c r="D11" s="4">
+      <c r="D11" s="3">
         <v>10</v>
       </c>
-      <c r="J11" s="4" t="s">
+      <c r="J11" s="3" t="s">
         <v>469</v>
       </c>
-      <c r="K11" s="4" t="s">
+      <c r="K11" s="3" t="s">
         <v>470</v>
       </c>
-      <c r="L11" s="4">
+      <c r="L11" s="3">
         <v>512</v>
       </c>
-      <c r="M11" s="4" t="s">
+      <c r="M11" s="3" t="s">
         <v>471</v>
       </c>
     </row>
     <row r="12" spans="2:13">
-      <c r="J12" s="4" t="s">
+      <c r="B12" t="s">
+        <v>418</v>
+      </c>
+      <c r="C12" t="s">
         <v>472</v>
       </c>
-      <c r="K12" s="4" t="s">
+      <c r="D12">
+        <v>11</v>
+      </c>
+      <c r="J12" s="3" t="s">
         <v>473</v>
       </c>
-      <c r="L12" s="4">
+      <c r="K12" s="3" t="s">
+        <v>474</v>
+      </c>
+      <c r="L12" s="3">
         <v>1024</v>
       </c>
-      <c r="M12" s="4" t="s">
-        <v>474</v>
+      <c r="M12" s="3" t="s">
+        <v>475</v>
       </c>
     </row>
     <row r="13" spans="2:13">
-      <c r="J13" s="4" t="s">
-        <v>475</v>
-      </c>
-      <c r="K13" s="4" t="s">
+      <c r="J13" s="3" t="s">
         <v>476</v>
       </c>
-      <c r="L13" s="4">
+      <c r="K13" s="3" t="s">
+        <v>477</v>
+      </c>
+      <c r="L13" s="3">
         <v>2048</v>
       </c>
-      <c r="M13" s="4" t="s">
-        <v>477</v>
+      <c r="M13" s="3" t="s">
+        <v>478</v>
       </c>
     </row>
   </sheetData>
@@ -6951,49 +6994,49 @@
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="I1" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="J1" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="K1" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="L1" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="M1" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="N1" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="O1" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="P1" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="Q1" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="R1" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
     </row>
     <row r="2" spans="1:18">
@@ -7058,10 +7101,10 @@
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
@@ -7074,52 +7117,52 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="D4" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="E4" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="F4" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="G4" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="H4" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="I4" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="J4" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="K4" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="L4" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="M4" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="N4" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="O4" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="P4" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="Q4" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="R4" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
     </row>
     <row r="5" spans="1:18">
@@ -7127,52 +7170,52 @@
         <v>1001</v>
       </c>
       <c r="C5" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="D5" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="E5" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="F5" t="s">
+        <v>514</v>
+      </c>
+      <c r="G5" t="s">
+        <v>515</v>
+      </c>
+      <c r="H5" t="s">
+        <v>516</v>
+      </c>
+      <c r="I5" t="s">
+        <v>517</v>
+      </c>
+      <c r="J5" t="s">
+        <v>518</v>
+      </c>
+      <c r="K5" t="s">
         <v>513</v>
       </c>
-      <c r="G5" t="s">
+      <c r="L5" t="s">
+        <v>519</v>
+      </c>
+      <c r="M5" t="s">
+        <v>520</v>
+      </c>
+      <c r="N5" t="s">
         <v>514</v>
       </c>
-      <c r="H5" t="s">
-        <v>515</v>
-      </c>
-      <c r="I5" t="s">
-        <v>516</v>
-      </c>
-      <c r="J5" t="s">
-        <v>517</v>
-      </c>
-      <c r="K5" t="s">
-        <v>512</v>
-      </c>
-      <c r="L5" t="s">
-        <v>518</v>
-      </c>
-      <c r="M5" t="s">
-        <v>519</v>
-      </c>
-      <c r="N5" t="s">
-        <v>513</v>
-      </c>
       <c r="O5" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="P5" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="Q5" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="R5" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="6" spans="1:18">
@@ -7183,49 +7226,49 @@
         <v>52</v>
       </c>
       <c r="D6" t="s">
+        <v>525</v>
+      </c>
+      <c r="E6" t="s">
+        <v>513</v>
+      </c>
+      <c r="F6" t="s">
+        <v>521</v>
+      </c>
+      <c r="G6" t="s">
+        <v>526</v>
+      </c>
+      <c r="H6" t="s">
+        <v>516</v>
+      </c>
+      <c r="I6" t="s">
+        <v>517</v>
+      </c>
+      <c r="J6" t="s">
+        <v>518</v>
+      </c>
+      <c r="K6" t="s">
+        <v>513</v>
+      </c>
+      <c r="L6" t="s">
+        <v>519</v>
+      </c>
+      <c r="M6" t="s">
+        <v>520</v>
+      </c>
+      <c r="N6" t="s">
+        <v>514</v>
+      </c>
+      <c r="O6" t="s">
+        <v>521</v>
+      </c>
+      <c r="P6" t="s">
+        <v>522</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>523</v>
+      </c>
+      <c r="R6" t="s">
         <v>524</v>
-      </c>
-      <c r="E6" t="s">
-        <v>512</v>
-      </c>
-      <c r="F6" t="s">
-        <v>520</v>
-      </c>
-      <c r="G6" t="s">
-        <v>525</v>
-      </c>
-      <c r="H6" t="s">
-        <v>515</v>
-      </c>
-      <c r="I6" t="s">
-        <v>516</v>
-      </c>
-      <c r="J6" t="s">
-        <v>517</v>
-      </c>
-      <c r="K6" t="s">
-        <v>512</v>
-      </c>
-      <c r="L6" t="s">
-        <v>518</v>
-      </c>
-      <c r="M6" t="s">
-        <v>519</v>
-      </c>
-      <c r="N6" t="s">
-        <v>513</v>
-      </c>
-      <c r="O6" t="s">
-        <v>520</v>
-      </c>
-      <c r="P6" t="s">
-        <v>521</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>522</v>
-      </c>
-      <c r="R6" t="s">
-        <v>523</v>
       </c>
     </row>
     <row r="7" spans="1:18">
@@ -7236,49 +7279,49 @@
         <v>56</v>
       </c>
       <c r="D7" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="E7" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="F7" t="s">
+        <v>522</v>
+      </c>
+      <c r="G7" t="s">
+        <v>528</v>
+      </c>
+      <c r="H7" t="s">
+        <v>516</v>
+      </c>
+      <c r="I7" t="s">
+        <v>517</v>
+      </c>
+      <c r="J7" t="s">
+        <v>518</v>
+      </c>
+      <c r="K7" t="s">
+        <v>513</v>
+      </c>
+      <c r="L7" t="s">
+        <v>519</v>
+      </c>
+      <c r="M7" t="s">
+        <v>520</v>
+      </c>
+      <c r="N7" t="s">
+        <v>514</v>
+      </c>
+      <c r="O7" t="s">
         <v>521</v>
       </c>
-      <c r="G7" t="s">
-        <v>527</v>
-      </c>
-      <c r="H7" t="s">
-        <v>515</v>
-      </c>
-      <c r="I7" t="s">
-        <v>516</v>
-      </c>
-      <c r="J7" t="s">
-        <v>517</v>
-      </c>
-      <c r="K7" t="s">
-        <v>512</v>
-      </c>
-      <c r="L7" t="s">
-        <v>518</v>
-      </c>
-      <c r="M7" t="s">
-        <v>519</v>
-      </c>
-      <c r="N7" t="s">
-        <v>513</v>
-      </c>
-      <c r="O7" t="s">
-        <v>520</v>
-      </c>
       <c r="P7" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="Q7" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="R7" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="8" spans="1:18">
@@ -7289,49 +7332,49 @@
         <v>60</v>
       </c>
       <c r="D8" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="E8" t="s">
+        <v>519</v>
+      </c>
+      <c r="F8" t="s">
+        <v>520</v>
+      </c>
+      <c r="G8" t="s">
+        <v>530</v>
+      </c>
+      <c r="H8" t="s">
+        <v>516</v>
+      </c>
+      <c r="I8" t="s">
+        <v>517</v>
+      </c>
+      <c r="J8" t="s">
         <v>518</v>
       </c>
-      <c r="F8" t="s">
+      <c r="K8" t="s">
+        <v>513</v>
+      </c>
+      <c r="L8" t="s">
         <v>519</v>
       </c>
-      <c r="G8" t="s">
-        <v>529</v>
-      </c>
-      <c r="H8" t="s">
-        <v>515</v>
-      </c>
-      <c r="I8" t="s">
-        <v>516</v>
-      </c>
-      <c r="J8" t="s">
-        <v>517</v>
-      </c>
-      <c r="K8" t="s">
-        <v>512</v>
-      </c>
-      <c r="L8" t="s">
-        <v>518</v>
-      </c>
       <c r="M8" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="N8" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="O8" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="P8" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="Q8" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="R8" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="9" spans="1:18">
@@ -7342,49 +7385,49 @@
         <v>64</v>
       </c>
       <c r="D9" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="E9" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="F9" t="s">
+        <v>522</v>
+      </c>
+      <c r="G9" t="s">
+        <v>515</v>
+      </c>
+      <c r="H9" t="s">
+        <v>532</v>
+      </c>
+      <c r="I9" t="s">
+        <v>517</v>
+      </c>
+      <c r="J9" t="s">
+        <v>518</v>
+      </c>
+      <c r="K9" t="s">
+        <v>513</v>
+      </c>
+      <c r="L9" t="s">
+        <v>519</v>
+      </c>
+      <c r="M9" t="s">
+        <v>520</v>
+      </c>
+      <c r="N9" t="s">
+        <v>514</v>
+      </c>
+      <c r="O9" t="s">
         <v>521</v>
       </c>
-      <c r="G9" t="s">
-        <v>514</v>
-      </c>
-      <c r="H9" t="s">
-        <v>531</v>
-      </c>
-      <c r="I9" t="s">
-        <v>516</v>
-      </c>
-      <c r="J9" t="s">
-        <v>517</v>
-      </c>
-      <c r="K9" t="s">
-        <v>512</v>
-      </c>
-      <c r="L9" t="s">
-        <v>518</v>
-      </c>
-      <c r="M9" t="s">
-        <v>519</v>
-      </c>
-      <c r="N9" t="s">
-        <v>513</v>
-      </c>
-      <c r="O9" t="s">
-        <v>520</v>
-      </c>
       <c r="P9" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="Q9" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="R9" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="10" spans="1:18">
@@ -7395,49 +7438,49 @@
         <v>68</v>
       </c>
       <c r="D10" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="E10" t="s">
+        <v>519</v>
+      </c>
+      <c r="F10" t="s">
+        <v>514</v>
+      </c>
+      <c r="G10" t="s">
+        <v>515</v>
+      </c>
+      <c r="H10" t="s">
+        <v>534</v>
+      </c>
+      <c r="I10" t="s">
+        <v>517</v>
+      </c>
+      <c r="J10" t="s">
         <v>518</v>
       </c>
-      <c r="F10" t="s">
+      <c r="K10" t="s">
         <v>513</v>
       </c>
-      <c r="G10" t="s">
+      <c r="L10" t="s">
+        <v>519</v>
+      </c>
+      <c r="M10" t="s">
+        <v>520</v>
+      </c>
+      <c r="N10" t="s">
         <v>514</v>
       </c>
-      <c r="H10" t="s">
-        <v>533</v>
-      </c>
-      <c r="I10" t="s">
-        <v>516</v>
-      </c>
-      <c r="J10" t="s">
-        <v>517</v>
-      </c>
-      <c r="K10" t="s">
-        <v>512</v>
-      </c>
-      <c r="L10" t="s">
-        <v>518</v>
-      </c>
-      <c r="M10" t="s">
-        <v>519</v>
-      </c>
-      <c r="N10" t="s">
-        <v>513</v>
-      </c>
       <c r="O10" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="P10" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="Q10" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="R10" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="11" spans="1:18">
@@ -7448,49 +7491,49 @@
         <v>71</v>
       </c>
       <c r="D11" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="E11" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="F11" t="s">
+        <v>524</v>
+      </c>
+      <c r="G11" t="s">
+        <v>526</v>
+      </c>
+      <c r="H11" t="s">
+        <v>532</v>
+      </c>
+      <c r="I11" t="s">
+        <v>517</v>
+      </c>
+      <c r="J11" t="s">
+        <v>518</v>
+      </c>
+      <c r="K11" t="s">
+        <v>513</v>
+      </c>
+      <c r="L11" t="s">
+        <v>519</v>
+      </c>
+      <c r="M11" t="s">
+        <v>520</v>
+      </c>
+      <c r="N11" t="s">
+        <v>514</v>
+      </c>
+      <c r="O11" t="s">
+        <v>521</v>
+      </c>
+      <c r="P11" t="s">
+        <v>522</v>
+      </c>
+      <c r="Q11" t="s">
         <v>523</v>
       </c>
-      <c r="G11" t="s">
-        <v>525</v>
-      </c>
-      <c r="H11" t="s">
-        <v>531</v>
-      </c>
-      <c r="I11" t="s">
-        <v>516</v>
-      </c>
-      <c r="J11" t="s">
-        <v>517</v>
-      </c>
-      <c r="K11" t="s">
-        <v>512</v>
-      </c>
-      <c r="L11" t="s">
-        <v>518</v>
-      </c>
-      <c r="M11" t="s">
-        <v>519</v>
-      </c>
-      <c r="N11" t="s">
-        <v>513</v>
-      </c>
-      <c r="O11" t="s">
-        <v>520</v>
-      </c>
-      <c r="P11" t="s">
-        <v>521</v>
-      </c>
-      <c r="Q11" t="s">
-        <v>522</v>
-      </c>
       <c r="R11" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="12" spans="1:18">
@@ -7501,49 +7544,49 @@
         <v>74</v>
       </c>
       <c r="D12" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="E12" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="F12" t="s">
+        <v>514</v>
+      </c>
+      <c r="G12" t="s">
+        <v>526</v>
+      </c>
+      <c r="H12" t="s">
+        <v>534</v>
+      </c>
+      <c r="I12" t="s">
+        <v>517</v>
+      </c>
+      <c r="J12" t="s">
+        <v>518</v>
+      </c>
+      <c r="K12" t="s">
         <v>513</v>
       </c>
-      <c r="G12" t="s">
-        <v>525</v>
-      </c>
-      <c r="H12" t="s">
-        <v>533</v>
-      </c>
-      <c r="I12" t="s">
-        <v>516</v>
-      </c>
-      <c r="J12" t="s">
-        <v>517</v>
-      </c>
-      <c r="K12" t="s">
-        <v>512</v>
-      </c>
       <c r="L12" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="M12" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="N12" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="O12" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="P12" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="Q12" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="R12" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="13" spans="1:18">
@@ -7554,49 +7597,49 @@
         <v>77</v>
       </c>
       <c r="D13" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="E13" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="F13" t="s">
+        <v>524</v>
+      </c>
+      <c r="G13" t="s">
+        <v>528</v>
+      </c>
+      <c r="H13" t="s">
+        <v>532</v>
+      </c>
+      <c r="I13" t="s">
+        <v>517</v>
+      </c>
+      <c r="J13" t="s">
+        <v>518</v>
+      </c>
+      <c r="K13" t="s">
+        <v>513</v>
+      </c>
+      <c r="L13" t="s">
+        <v>519</v>
+      </c>
+      <c r="M13" t="s">
+        <v>520</v>
+      </c>
+      <c r="N13" t="s">
+        <v>514</v>
+      </c>
+      <c r="O13" t="s">
+        <v>521</v>
+      </c>
+      <c r="P13" t="s">
+        <v>522</v>
+      </c>
+      <c r="Q13" t="s">
         <v>523</v>
       </c>
-      <c r="G13" t="s">
-        <v>527</v>
-      </c>
-      <c r="H13" t="s">
-        <v>531</v>
-      </c>
-      <c r="I13" t="s">
-        <v>516</v>
-      </c>
-      <c r="J13" t="s">
-        <v>517</v>
-      </c>
-      <c r="K13" t="s">
-        <v>512</v>
-      </c>
-      <c r="L13" t="s">
-        <v>518</v>
-      </c>
-      <c r="M13" t="s">
-        <v>519</v>
-      </c>
-      <c r="N13" t="s">
-        <v>513</v>
-      </c>
-      <c r="O13" t="s">
-        <v>520</v>
-      </c>
-      <c r="P13" t="s">
-        <v>521</v>
-      </c>
-      <c r="Q13" t="s">
-        <v>522</v>
-      </c>
       <c r="R13" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="14" spans="1:18">
@@ -7607,49 +7650,49 @@
         <v>80</v>
       </c>
       <c r="D14" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="E14" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="F14" t="s">
+        <v>514</v>
+      </c>
+      <c r="G14" t="s">
+        <v>528</v>
+      </c>
+      <c r="H14" t="s">
+        <v>534</v>
+      </c>
+      <c r="I14" t="s">
+        <v>517</v>
+      </c>
+      <c r="J14" t="s">
+        <v>518</v>
+      </c>
+      <c r="K14" t="s">
         <v>513</v>
       </c>
-      <c r="G14" t="s">
-        <v>527</v>
-      </c>
-      <c r="H14" t="s">
-        <v>533</v>
-      </c>
-      <c r="I14" t="s">
-        <v>516</v>
-      </c>
-      <c r="J14" t="s">
-        <v>517</v>
-      </c>
-      <c r="K14" t="s">
-        <v>512</v>
-      </c>
       <c r="L14" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="M14" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="N14" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="O14" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="P14" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="Q14" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="R14" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="15" spans="1:18">
@@ -7660,49 +7703,49 @@
         <v>83</v>
       </c>
       <c r="D15" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="E15" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="F15" t="s">
+        <v>514</v>
+      </c>
+      <c r="G15" t="s">
+        <v>530</v>
+      </c>
+      <c r="H15" t="s">
+        <v>532</v>
+      </c>
+      <c r="I15" t="s">
+        <v>517</v>
+      </c>
+      <c r="J15" t="s">
+        <v>518</v>
+      </c>
+      <c r="K15" t="s">
         <v>513</v>
       </c>
-      <c r="G15" t="s">
-        <v>529</v>
-      </c>
-      <c r="H15" t="s">
-        <v>531</v>
-      </c>
-      <c r="I15" t="s">
-        <v>516</v>
-      </c>
-      <c r="J15" t="s">
-        <v>517</v>
-      </c>
-      <c r="K15" t="s">
-        <v>512</v>
-      </c>
       <c r="L15" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="M15" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="N15" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="O15" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="P15" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="Q15" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="R15" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
     <row r="16" spans="1:18">
@@ -7710,52 +7753,52 @@
         <v>1012</v>
       </c>
       <c r="C16" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="D16" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="E16" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="F16" t="s">
+        <v>523</v>
+      </c>
+      <c r="G16" t="s">
+        <v>530</v>
+      </c>
+      <c r="H16" t="s">
+        <v>534</v>
+      </c>
+      <c r="I16" t="s">
+        <v>517</v>
+      </c>
+      <c r="J16" t="s">
+        <v>518</v>
+      </c>
+      <c r="K16" t="s">
+        <v>513</v>
+      </c>
+      <c r="L16" t="s">
+        <v>519</v>
+      </c>
+      <c r="M16" t="s">
+        <v>520</v>
+      </c>
+      <c r="N16" t="s">
+        <v>514</v>
+      </c>
+      <c r="O16" t="s">
+        <v>521</v>
+      </c>
+      <c r="P16" t="s">
         <v>522</v>
       </c>
-      <c r="G16" t="s">
-        <v>529</v>
-      </c>
-      <c r="H16" t="s">
-        <v>533</v>
-      </c>
-      <c r="I16" t="s">
-        <v>516</v>
-      </c>
-      <c r="J16" t="s">
-        <v>517</v>
-      </c>
-      <c r="K16" t="s">
-        <v>512</v>
-      </c>
-      <c r="L16" t="s">
-        <v>518</v>
-      </c>
-      <c r="M16" t="s">
-        <v>519</v>
-      </c>
-      <c r="N16" t="s">
-        <v>513</v>
-      </c>
-      <c r="O16" t="s">
-        <v>520</v>
-      </c>
-      <c r="P16" t="s">
-        <v>521</v>
-      </c>
       <c r="Q16" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="R16" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
     </row>
   </sheetData>
@@ -7783,10 +7826,10 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="D1" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="E1" t="s">
         <v>12</v>
@@ -7800,7 +7843,7 @@
         <v>15</v>
       </c>
       <c r="C2" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="D2" t="s">
         <v>15</v>
@@ -7817,12 +7860,12 @@
         <v>32</v>
       </c>
       <c r="C3" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="D3" t="s">
-        <v>545</v>
-      </c>
-      <c r="E3" s="3" t="s">
+        <v>546</v>
+      </c>
+      <c r="E3" s="4" t="s">
         <v>42</v>
       </c>
     </row>
@@ -7920,60 +7963,60 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="5" t="s">
-        <v>546</v>
-      </c>
-      <c r="B1" s="4" t="s">
+        <v>547</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4" t="s">
+      <c r="D1" s="3"/>
+      <c r="E1" s="3" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="5"/>
-      <c r="B2" s="4" t="s">
-        <v>547</v>
-      </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>548</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="C2" s="3"/>
+      <c r="D2" s="3" t="s">
         <v>549</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>550</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="1" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>551</v>
-      </c>
-      <c r="C3" s="4" t="s">
+        <v>552</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>19</v>
       </c>
       <c r="D3" s="1" t="b">
         <v>0</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
-      <c r="C4" s="4"/>
+      <c r="C4" s="3"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="1"/>
       <c r="B5" s="1"/>
-      <c r="C5" s="4"/>
+      <c r="C5" s="3"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
     </row>
@@ -7986,7 +8029,7 @@
     <row r="7" spans="1:5">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
-      <c r="C7" s="4"/>
+      <c r="C7" s="3"/>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
     </row>
@@ -7999,7 +8042,7 @@
     <row r="9" spans="1:5">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
-      <c r="C9" s="4"/>
+      <c r="C9" s="3"/>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
     </row>
@@ -8011,14 +8054,14 @@
     <row r="11" spans="1:5">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
-      <c r="C11" s="4"/>
+      <c r="C11" s="3"/>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
     </row>
     <row r="12" spans="1:5">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
-      <c r="C12" s="4"/>
+      <c r="C12" s="3"/>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
     </row>
@@ -8048,16 +8091,16 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="E1" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="F1" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -8095,16 +8138,16 @@
         <v>32</v>
       </c>
       <c r="C4" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="D4" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="E4" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="F4" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -8115,13 +8158,13 @@
         <v>50</v>
       </c>
       <c r="D5" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="E5" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="F5" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -8132,13 +8175,13 @@
         <v>100</v>
       </c>
       <c r="D6" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="E6" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="F6" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -8149,13 +8192,13 @@
         <v>150</v>
       </c>
       <c r="D7" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="E7" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="F7" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -8166,13 +8209,13 @@
         <v>200</v>
       </c>
       <c r="D8" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="E8" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="F8" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -8183,13 +8226,13 @@
         <v>300</v>
       </c>
       <c r="D9" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="E9" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="F9" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -8200,13 +8243,13 @@
         <v>450</v>
       </c>
       <c r="D10" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="E10" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="F10" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -8217,13 +8260,13 @@
         <v>1000</v>
       </c>
       <c r="D11" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="E11" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="F11" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -8234,13 +8277,13 @@
         <v>2500</v>
       </c>
       <c r="D12" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E12" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="F12" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -8251,13 +8294,13 @@
         <v>12500</v>
       </c>
       <c r="D13" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="E13" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="F13" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
     </row>
   </sheetData>
@@ -8292,10 +8335,10 @@
         <v>4</v>
       </c>
       <c r="E1" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="F1" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -8324,7 +8367,7 @@
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
-      <c r="D3" s="3"/>
+      <c r="D3" s="4"/>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" t="s">
@@ -8340,113 +8383,330 @@
         <v>36</v>
       </c>
       <c r="E4" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="F4" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="B5">
         <v>1001</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="3" t="s">
         <v>426</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="3" t="s">
         <v>65</v>
       </c>
       <c r="E5" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="F5" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="B6">
         <v>1002</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="3" t="s">
         <v>430</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="3" t="s">
         <v>48</v>
       </c>
       <c r="E6" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="F6" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="B7">
         <v>1003</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="3" t="s">
         <v>435</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="3" t="s">
         <v>91</v>
       </c>
       <c r="E7" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="F7" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="B8">
         <v>1004</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="3" t="s">
         <v>440</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="3" t="s">
         <v>366</v>
       </c>
       <c r="E8" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="F8" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="B9">
         <v>1005</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="3" t="s">
         <v>445</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="3" t="s">
         <v>446</v>
       </c>
       <c r="E9" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="F9" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="B10">
         <v>1006</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="3" t="s">
         <v>451</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="3" t="s">
         <v>452</v>
       </c>
       <c r="E10" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="F10" t="s">
-        <v>603</v>
-      </c>
+        <v>604</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:E32"/>
+  <sheetFormatPr defaultColWidth="8.66666666666667" defaultRowHeight="17.4" outlineLevelCol="4"/>
+  <cols>
+    <col min="3" max="3" width="13.5" customWidth="1"/>
+    <col min="4" max="4" width="21.8333333333333" customWidth="1"/>
+    <col min="5" max="5" width="13.25" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>605</v>
+      </c>
+      <c r="D1" t="s">
+        <v>606</v>
+      </c>
+      <c r="E1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" t="s">
+        <v>607</v>
+      </c>
+      <c r="E2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" t="s">
+        <v>608</v>
+      </c>
+      <c r="E3" t="s">
+        <v>609</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="B4">
+        <v>1001</v>
+      </c>
+      <c r="C4" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="B5">
+        <v>1002</v>
+      </c>
+      <c r="C5" t="s">
+        <v>610</v>
+      </c>
+      <c r="D5" t="s">
+        <v>90</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="B6">
+        <v>1003</v>
+      </c>
+      <c r="C6" t="s">
+        <v>611</v>
+      </c>
+      <c r="D6" t="s">
+        <v>132</v>
+      </c>
+      <c r="E6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="B7">
+        <v>1004</v>
+      </c>
+      <c r="C7" t="s">
+        <v>612</v>
+      </c>
+      <c r="D7" t="s">
+        <v>153</v>
+      </c>
+      <c r="E7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="D8" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="D9" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="B10">
+        <v>1005</v>
+      </c>
+      <c r="C10" t="s">
+        <v>613</v>
+      </c>
+      <c r="D10" t="s">
+        <v>204</v>
+      </c>
+      <c r="E10">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="D11" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="D12" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="B13">
+        <v>1006</v>
+      </c>
+      <c r="C13" t="s">
+        <v>614</v>
+      </c>
+      <c r="D13" t="s">
+        <v>413</v>
+      </c>
+      <c r="E13">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="D14" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="23" spans="3:4">
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+    </row>
+    <row r="24" spans="3:4">
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+    </row>
+    <row r="25" spans="3:4">
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+    </row>
+    <row r="26" spans="3:4">
+      <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
+    </row>
+    <row r="27" spans="3:4">
+      <c r="C27" s="3"/>
+      <c r="D27" s="3"/>
+    </row>
+    <row r="28" spans="3:4">
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+    </row>
+    <row r="29" spans="3:4">
+      <c r="C29" s="3"/>
+      <c r="D29" s="3"/>
+    </row>
+    <row r="30" spans="3:4">
+      <c r="C30" s="3"/>
+      <c r="D30" s="3"/>
+    </row>
+    <row r="31" spans="3:4">
+      <c r="C31" s="3"/>
+      <c r="D31" s="3"/>
+    </row>
+    <row r="32" spans="3:4">
+      <c r="C32" s="3"/>
+      <c r="D32" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>